<commit_message>
Add Ultimate Christmas Organiser bundle; switch templates to GBP
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XAZTcsRbYDYsZphEU6c43B
</commit_message>
<xml_diff>
--- a/etsy-templates/Budget-Planner.xlsx
+++ b/etsy-templates/Budget-Planner.xlsx
@@ -304,7 +304,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="mmm\ yyyy"/>
     <numFmt numFmtId="166" formatCode="dd\ mmm\ yyyy"/>
-    <numFmt numFmtId="167" formatCode="\$#,##0.00;&quot;-$&quot;#,##0.00;\-"/>
+    <numFmt numFmtId="167" formatCode="\£#,##0.00;&quot;-£&quot;#,##0.00;\-"/>
     <numFmt numFmtId="168" formatCode="0%"/>
     <numFmt numFmtId="169" formatCode="#,##0;\-#,##0;\-"/>
   </numFmts>
@@ -912,7 +912,7 @@
             <c:numRef>
               <c:f>Budget!$C$17:$C$32</c:f>
               <c:numCache>
-                <c:formatCode>\$#,##0.00;"-$"#,##0.00;\-</c:formatCode>
+                <c:formatCode>\£#,##0.00;"-£"#,##0.00;\-</c:formatCode>
                 <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>1100</c:v>
@@ -1077,7 +1077,7 @@
             <c:numRef>
               <c:f>Budget!$D$17:$D$32</c:f>
               <c:numCache>
-                <c:formatCode>\$#,##0.00;"-$"#,##0.00;\-</c:formatCode>
+                <c:formatCode>\£#,##0.00;"-£"#,##0.00;\-</c:formatCode>
                 <c:ptCount val="16"/>
                 <c:pt idx="0">
                   <c:v>1100</c:v>
@@ -1133,11 +1133,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="27771492"/>
-        <c:axId val="40327180"/>
+        <c:axId val="95563447"/>
+        <c:axId val="72971196"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="27771492"/>
+        <c:axId val="95563447"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1169,7 +1169,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40327180"/>
+        <c:crossAx val="72971196"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1177,13 +1177,13 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="40327180"/>
+        <c:axId val="72971196"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:numFmt formatCode="\$#,##0.00;&quot;-$&quot;#,##0.00;\-" sourceLinked="1"/>
+        <c:numFmt formatCode="\£#,##0.00;&quot;-£&quot;#,##0.00;\-" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1209,7 +1209,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27771492"/>
+        <c:crossAx val="95563447"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2141,7 +2141,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7457C827-F81E-48B0-AAE3-50B0F04D14C4}</x14:id>
+          <x14:id>{FBA27BA0-2F56-44EC-ADEF-AD8384ADEC78}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -2164,7 +2164,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7457C827-F81E-48B0-AAE3-50B0F04D14C4}">
+          <x14:cfRule type="dataBar" id="{FBA27BA0-2F56-44EC-ADEF-AD8384ADEC78}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>